<commit_message>
auto update queens news 2026-09-08T16:35:14Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,74 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>JCS Realty Group files plans for 495 units in LIC, Acris does not yet show JCS as owner</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/jcs-realty-group-files-plans-for-495-units-in-lic-no-sale-lease-to-developer-yet-in-acris/</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Jacob Schwimmer of JCS Realty Group filed plans last week for five buildings with a</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Development 45-03 Vernon Boulevard, 10-24 45th Avenue, 10-26 45th Avenue, 10-27 45th Road, 10-25 45th Road (Credit - Google Earth) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Joel Teitelbaum, Shimon Brach pay $28.5M to Mitsubishi for office, retail in Williamsburg</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/joel-teitelbaum-shimon-brach-pay-28-5m-to-mitsubishi-for-office-retail-in-williamsburg/</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Joel Teitelbaum and Shimon Brach paid $28.5 million to the Mitsubishi Corporation’s Diamond Realty Investments,</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Top Story Transfers 209 Havemeyer Street, aka 277 South 5th Street (Credit - Cyclomedia) Joel Teitelbaum and Shimon Brach paid $28.5 million to the Mitsubishi Corporation’s Diamond Realty Investments, for office and retail condominium units at 209 Havermeyer Street in Williamsburg, Brooklyn, in two transactions, borrowing $20 million to finance the purchase. The property is also known as 277 South 5th Street. In the office portion, Joel Teitelbaum and Shimon Brach through the entity Dime Commercial Holdings LLC paid $20.5 million to Mitsubishi Corporation through the entity Havemeyer Owner LLC for the office condominium units. The expected use is cash flowing. The deal closed on August 24, 2026 and was recorded on September 4, 2026. The three properties have 87,320 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $234 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Mitsubishi Corporation was Anthony Strauser . The signatory for Joel Teitelbaum and Shimon Brach was Jo</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-09-09T16:35:16Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,74 +467,6 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>JCS Realty Group files plans for 495 units in LIC, Acris does not yet show JCS as owner</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/jcs-realty-group-files-plans-for-495-units-in-lic-no-sale-lease-to-developer-yet-in-acris/</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Jacob Schwimmer of JCS Realty Group filed plans last week for five buildings with a</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Development 45-03 Vernon Boulevard, 10-24 45th Avenue, 10-26 45th Avenue, 10-27 45th Road, 10-25 45th Road (Credit - Google Earth) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Joel Teitelbaum, Shimon Brach pay $28.5M to Mitsubishi for office, retail in Williamsburg</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/joel-teitelbaum-shimon-brach-pay-28-5m-to-mitsubishi-for-office-retail-in-williamsburg/</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Joel Teitelbaum and Shimon Brach paid $28.5 million to the Mitsubishi Corporation’s Diamond Realty Investments,</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Top Story Transfers 209 Havemeyer Street, aka 277 South 5th Street (Credit - Cyclomedia) Joel Teitelbaum and Shimon Brach paid $28.5 million to the Mitsubishi Corporation’s Diamond Realty Investments, for office and retail condominium units at 209 Havermeyer Street in Williamsburg, Brooklyn, in two transactions, borrowing $20 million to finance the purchase. The property is also known as 277 South 5th Street. In the office portion, Joel Teitelbaum and Shimon Brach through the entity Dime Commercial Holdings LLC paid $20.5 million to Mitsubishi Corporation through the entity Havemeyer Owner LLC for the office condominium units. The expected use is cash flowing. The deal closed on August 24, 2026 and was recorded on September 4, 2026. The three properties have 87,320 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $234 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Mitsubishi Corporation was Anthony Strauser . The signatory for Joel Teitelbaum and Shimon Brach was Jo</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-09-10T16:21:24Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,74 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Marvan Properteis files plans for 44 units in Long Island City</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/marios-mouzouris-files-plans-for-44-units-in-long-island-city/</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Marios Mouzouris of Marvan Properties submitted a new building construction project for a 44-unit, 29,995-square-foot</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Development 41-14 and 41-16 29th Street axonometrict diagram (Credit - Harriet Nikakis architect via DOB) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Guan Yu Li seeks zoning changes to build 168-unit project in College Point</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/guan-yu-li-seeks-zoning-changes-to-build-168-unit-project-in-college-point/</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Guan Yu Li, through the entity Lee 28th Avenue Realty LLC, filed a land use</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Development 26-35 123rd Street ULURP project, red is development site, green is wider rezoning "project area" (Credit - Google Earth) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-09-11T16:25:13Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,74 +467,6 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Marvan Properteis files plans for 44 units in Long Island City</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/marios-mouzouris-files-plans-for-44-units-in-long-island-city/</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Marios Mouzouris of Marvan Properties submitted a new building construction project for a 44-unit, 29,995-square-foot</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Development 41-14 and 41-16 29th Street axonometrict diagram (Credit - Harriet Nikakis architect via DOB) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Guan Yu Li seeks zoning changes to build 168-unit project in College Point</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/guan-yu-li-seeks-zoning-changes-to-build-168-unit-project-in-college-point/</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Guan Yu Li, through the entity Lee 28th Avenue Realty LLC, filed a land use</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Development 26-35 123rd Street ULURP project, red is development site, green is wider rezoning "project area" (Credit - Google Earth) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-09-13T16:13:09Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,48 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Permits Filed for 41-14 29th Street in Astoria, Queens</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://newyorkyimby.com/2026/09/permits-filed-for-41-14-29th-street-in-astoria-queens.html</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Permits have been filed for a 13-story residential building at 41-14 29th Street in &lt;a href="https://newyorkyimby.com/neighborhoods/astoria"&gt;Astoria&lt;/a&gt;, Queens. Located between Queens Plaza North and 41st Avenue, the lot is near the Queens Plaza subway station, served by the E, F, and R trains. Marios Mouzouris of Marvan Properties Inc. is listed as the owner behind the applications.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-09-13T10:30:18+00:00</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Sun, 13 Sep 2026 10:30:18 +0000</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>YIMBY</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>YIMBY - Astoria</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>By: Vanessa Londono 6:30 am on September 13, 2026 Permits have been filed for a 13-story residential building at 41-14 29th Street in Astoria, Queens. Located between Queens Plaza North and 41st Avenue, the lot is near the Queens Plaza subway station, served by the E, F, and R trains. Marios Mouzouris of Marvan Properties Inc. is listed as the owner behind the applications. The proposed 135-foot-tall development will yield 29,995 square feet designated for residential space. The building will have 44 residences, most likely rentals based on the average unit scope of 681 square feet. The concrete-based structure will also have a cellar and a 37-foot-long rear yard. Harriet Nikakis of HCN Design is listed as the architect of record. Demolition permits have not been filed yet. An estimated completion date has not been announced. Subscribe to YIMBY’s daily e-mail Follow YIMBYgram for real-time photo updates Like YIMBY on Facebook Follow YIMBY’s Twitter for the latest in YIMBYnews</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-09-14T18:04:07Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,27 +473,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Permits Filed for 41-14 29th Street in Astoria, Queens</t>
+          <t>Permits Filed for 29-16 12th Street in Astoria, Queens</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://newyorkyimby.com/2026/09/permits-filed-for-41-14-29th-street-in-astoria-queens.html</t>
+          <t>https://newyorkyimby.com/2026/09/permits-filed-for-29-16-12th-street-in-astoria-queens.html</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Permits have been filed for a 13-story residential building at 41-14 29th Street in &lt;a href="https://newyorkyimby.com/neighborhoods/astoria"&gt;Astoria&lt;/a&gt;, Queens. Located between Queens Plaza North and 41st Avenue, the lot is near the Queens Plaza subway station, served by the E, F, and R trains. Marios Mouzouris of Marvan Properties Inc. is listed as the owner behind the applications.</t>
+          <t>Permits have been filed for a seven-story residential building at 29-16 12th Street in &lt;a href="https://newyorkyimby.com/neighborhoods/astoria"&gt;Astoria&lt;/a&gt;, Queens. Located between 29th Avenue and 30th Avenue, the corner lot is also addressed as 8-48 Astoria Boulevard. The closest public transit is 30th Avenue subway station, served by the N and W trains. Oleg Krasnitskiy is listed as the owner behind the applications.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-09-13T10:30:18+00:00</t>
+          <t>2026-09-14T10:30:04+00:00</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Sun, 13 Sep 2026 10:30:18 +0000</t>
+          <t>Mon, 14 Sep 2026 10:30:04 +0000</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -508,7 +508,45 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>By: Vanessa Londono 6:30 am on September 13, 2026 Permits have been filed for a 13-story residential building at 41-14 29th Street in Astoria, Queens. Located between Queens Plaza North and 41st Avenue, the lot is near the Queens Plaza subway station, served by the E, F, and R trains. Marios Mouzouris of Marvan Properties Inc. is listed as the owner behind the applications. The proposed 135-foot-tall development will yield 29,995 square feet designated for residential space. The building will have 44 residences, most likely rentals based on the average unit scope of 681 square feet. The concrete-based structure will also have a cellar and a 37-foot-long rear yard. Harriet Nikakis of HCN Design is listed as the architect of record. Demolition permits have not been filed yet. An estimated completion date has not been announced. Subscribe to YIMBY’s daily e-mail Follow YIMBYgram for real-time photo updates Like YIMBY on Facebook Follow YIMBY’s Twitter for the latest in YIMBYnews</t>
+          <t>By: Vanessa Londono 6:30 am on September 14, 2026 Permits have been filed for a seven-story residential building at 29-16 12th Street in Astoria, Queens. Located between 29th Avenue and 30th Avenue, the corner lot is also addressed as 8-48 Astoria Boulevard. The closest public transit is 30th Avenue subway station, served by the N and W trains. Oleg Krasnitskiy is listed as the owner behind the applications. The proposed 75-foot-tall development will yield 16,230 square feet designated for residential space. The building will have 24 residences, most likely rentals based on the average unit scope of 676 square feet. The concrete-based structure will also have a cellar but no accessory parking. Joseph Spector of Dome Architecture, Design &amp; Engineering is listed as the architect of record. Demolition permits will likely not be needed as the lot is vacant. An estimated completion date has not been announced. Subscribe to YIMBY’s daily e-mail Follow YIMBYgram for real-time photo updates Like YIMBY on Facebook Follow YIMBY’s Twitter for the latest in YIMBYnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Borrower seeks to block tomorrow’s $60.25M UCC foreclosure at 143-unit Astoria building</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/borrower-seeks-to-block-tomorrows-60-25m-ucc-foreclosure-at-118-unit-astoria-rental/</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Developer Sophia Shanfen Zhang and her associated entities filed a lawsuit in Queens County Supreme</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>NaT</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Transfers 26-01 4th Street (Credit - Cyclomedia) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-09-15T16:54:37Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -473,27 +473,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Permits Filed for 29-16 12th Street in Astoria, Queens</t>
+          <t>Permits Filed for 43-27 56th Street in Woodside, Queens</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://newyorkyimby.com/2026/09/permits-filed-for-29-16-12th-street-in-astoria-queens.html</t>
+          <t>https://newyorkyimby.com/2026/09/permits-filed-for-43-27-56th-street-in-woodside-queens-2.html</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Permits have been filed for a seven-story residential building at 29-16 12th Street in &lt;a href="https://newyorkyimby.com/neighborhoods/astoria"&gt;Astoria&lt;/a&gt;, Queens. Located between 29th Avenue and 30th Avenue, the corner lot is also addressed as 8-48 Astoria Boulevard. The closest public transit is 30th Avenue subway station, served by the N and W trains. Oleg Krasnitskiy is listed as the owner behind the applications.</t>
+          <t>Permits have been filed for a nine-story mixed-use building at 43-27 56th Street in &lt;a href="https://newyorkyimby.com/neighborhoods/sunnyside"&gt;Sunnyside&lt;/a&gt;, Queens. Located between 43rd Avenue and Queens Boulevard, the lot is near the 52nd Street subway station, served by the 7 train. Markiel Chulpayev is listed as the owner behind the applications.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-09-14T10:30:04+00:00</t>
+          <t>2026-09-15T10:30:11+00:00</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Mon, 14 Sep 2026 10:30:04 +0000</t>
+          <t>Tue, 15 Sep 2026 10:30:11 +0000</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -503,29 +503,29 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>YIMBY - Astoria</t>
+          <t>YIMBY - Sunnyside</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>By: Vanessa Londono 6:30 am on September 14, 2026 Permits have been filed for a seven-story residential building at 29-16 12th Street in Astoria, Queens. Located between 29th Avenue and 30th Avenue, the corner lot is also addressed as 8-48 Astoria Boulevard. The closest public transit is 30th Avenue subway station, served by the N and W trains. Oleg Krasnitskiy is listed as the owner behind the applications. The proposed 75-foot-tall development will yield 16,230 square feet designated for residential space. The building will have 24 residences, most likely rentals based on the average unit scope of 676 square feet. The concrete-based structure will also have a cellar but no accessory parking. Joseph Spector of Dome Architecture, Design &amp; Engineering is listed as the architect of record. Demolition permits will likely not be needed as the lot is vacant. An estimated completion date has not been announced. Subscribe to YIMBY’s daily e-mail Follow YIMBYgram for real-time photo updates Like YIMBY on Facebook Follow YIMBY’s Twitter for the latest in YIMBYnews</t>
+          <t>By: Vanessa Londono 6:30 am on September 15, 2026 Permits have been filed for a nine-story mixed-use building at 43-27 56th Street in Woodside, Queens. Located between 43rd Avenue and Queens Boulevard, the lot is near the 52nd Street subway station, served by the 7 train. Markiel Chulpayev is listed as the owner behind the applications. The proposed 116-foot-tall development will yield 22,922 square feet, with 21,905 square feet designated for residential space and 1,016 square feet for commercial space. The building will have 32 residences, most likely rentals based on the average unit scope of 684 square feet. The concrete-based structure will also have a cellar. Alexander Zhitnik of Z Architecture is listed as the architect of record. Demolition permits were filed last month for the single-story structure on the site. An estimated completion date has not been announced. Subscribe to YIMBY’s daily e-mail Follow YIMBYgram for real-time photo updates Like YIMBY on Facebook Follow YIMBY’s Twitter for the latest in YIMBYnews</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Borrower seeks to block tomorrow’s $60.25M UCC foreclosure at 143-unit Astoria building</t>
+          <t>Aaron Lebovits signs $50.4M construction loan with Ponce for development in Sunnyside</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/borrower-seeks-to-block-tomorrows-60-25m-ucc-foreclosure-at-118-unit-astoria-rental/</t>
+          <t>https://www.pincusco.com/aaron-lebovits-signs-50-4m-construction-loan-with-ponce-for-development-in-sunnyside/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Developer Sophia Shanfen Zhang and her associated entities filed a lawsuit in Queens County Supreme</t>
+          <t>Aaron Lebovits through the entity 42-25 Queens Blvd Holdings LLC as borrower signed a new</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -546,7 +546,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Transfers 26-01 4th Street (Credit - Cyclomedia) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
+          <t>Transfers 43-42 43rd Street axonometric diagram (Credit - Gerald Caliendo architect via DOB) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-09-16T16:49:24Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,86 +467,6 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Permits Filed for 43-27 56th Street in Woodside, Queens</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>https://newyorkyimby.com/2026/09/permits-filed-for-43-27-56th-street-in-woodside-queens-2.html</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Permits have been filed for a nine-story mixed-use building at 43-27 56th Street in &lt;a href="https://newyorkyimby.com/neighborhoods/sunnyside"&gt;Sunnyside&lt;/a&gt;, Queens. Located between 43rd Avenue and Queens Boulevard, the lot is near the 52nd Street subway station, served by the 7 train. Markiel Chulpayev is listed as the owner behind the applications.</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2026-09-15T10:30:11+00:00</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Tue, 15 Sep 2026 10:30:11 +0000</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>YIMBY</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>YIMBY - Sunnyside</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>By: Vanessa Londono 6:30 am on September 15, 2026 Permits have been filed for a nine-story mixed-use building at 43-27 56th Street in Woodside, Queens. Located between 43rd Avenue and Queens Boulevard, the lot is near the 52nd Street subway station, served by the 7 train. Markiel Chulpayev is listed as the owner behind the applications. The proposed 116-foot-tall development will yield 22,922 square feet, with 21,905 square feet designated for residential space and 1,016 square feet for commercial space. The building will have 32 residences, most likely rentals based on the average unit scope of 684 square feet. The concrete-based structure will also have a cellar. Alexander Zhitnik of Z Architecture is listed as the architect of record. Demolition permits were filed last month for the single-story structure on the site. An estimated completion date has not been announced. Subscribe to YIMBY’s daily e-mail Follow YIMBYgram for real-time photo updates Like YIMBY on Facebook Follow YIMBY’s Twitter for the latest in YIMBYnews</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Aaron Lebovits signs $50.4M construction loan with Ponce for development in Sunnyside</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/aaron-lebovits-signs-50-4m-construction-loan-with-ponce-for-development-in-sunnyside/</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Aaron Lebovits through the entity 42-25 Queens Blvd Holdings LLC as borrower signed a new</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>NaT</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Transfers 43-42 43rd Street axonometric diagram (Credit - Gerald Caliendo architect via DOB) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-09-17T16:56:40Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,40 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Ilias Theodoropoulos pays $4M for 17-apartment condo unit in Astoria</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/ilias-theodoropoulos-pays-4m-for-17-apartment-condo-unit-in-astoria/</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Ilias Theodoropoulos through the entity Amorani Square LLC paid $4 million to the entity 18-10</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Transfers Ilias Theodoropoulos through the entity Amorani Square LLC paid $4 million to the entity 18-10 LLC for the 17-apartment condominium unit at 18-10 27th Avenue in Astoria, Queens. The expected use is cash flowing. The deal closed on September 9, 2026 and was recorded on September 15, 2026. The property has 18,883 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $211 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for the seller was Benedetto Filingeri. The signatory for Ilias Theodoropoulos was Ilias Theodoropoulos. The contract date was May 21, 2026. The building is divided into a retail condo and the multi-unit residential condo. This purchase only involves the 17-unit residential condo unit. The 19,704-square-foot retail unit was not involved. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Ilias Theodoropoulos had purchased any other properties and has no record it sold any properties over the past 24 months.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-09-18T16:21:17Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -473,34 +473,42 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Ilias Theodoropoulos pays $4M for 17-apartment condo unit in Astoria</t>
+          <t>Permits Filed for 149-16 Archer Avenue in Jamaica, Queens</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/ilias-theodoropoulos-pays-4m-for-17-apartment-condo-unit-in-astoria/</t>
+          <t>https://newyorkyimby.com/2026/09/permits-filed-for-149-16-archer-avenue-in-jamaica-queens.html</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Ilias Theodoropoulos through the entity Amorani Square LLC paid $4 million to the entity 18-10</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
+          <t>Permits have been filed for a seven-story mixed-use building at 149-16 Archer Avenue in &lt;a href="https://newyorkyimby.com/neighborhoods/jamaica"&gt;Jamaica&lt;/a&gt;, Queens. Located between Sutphin Boulevard and 150th Street, the lot is near the Sutphin Blvd–Archer Avenue–JFK Airport subway station, served by the E, J, and Z trains. Shulem Rabi is listed as the owner behind the applications.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-09-18T10:30:55+00:00</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Fri, 18 Sep 2026 10:30:55 +0000</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>PincusCo</t>
+          <t>YIMBY</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>PincusCo - Home</t>
+          <t>YIMBY - Jamaica</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Transfers Ilias Theodoropoulos through the entity Amorani Square LLC paid $4 million to the entity 18-10 LLC for the 17-apartment condominium unit at 18-10 27th Avenue in Astoria, Queens. The expected use is cash flowing. The deal closed on September 9, 2026 and was recorded on September 15, 2026. The property has 18,883 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $211 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for the seller was Benedetto Filingeri. The signatory for Ilias Theodoropoulos was Ilias Theodoropoulos. The contract date was May 21, 2026. The building is divided into a retail condo and the multi-unit residential condo. This purchase only involves the 17-unit residential condo unit. The 19,704-square-foot retail unit was not involved. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Ilias Theodoropoulos had purchased any other properties and has no record it sold any properties over the past 24 months.</t>
+          <t>By: Vanessa Londono 6:30 am on September 18, 2026 Permits have been filed for a seven-story mixed-use building at 149-16 Archer Avenue in Jamaica, Queens. Located between Sutphin Boulevard and 150th Street, the lot is near the Sutphin Blvd–Archer Avenue–JFK Airport subway station, served by the E, J, and Z trains. Shulem Rabi is listed as the owner behind the applications. The proposed 70-foot-tall development will yield 27,127 square feet, with 25,304 square feet designated for residential space and 1,822 square feet for commercial space. The building will have 24 residences, most likely condos based on the average unit scope of 1,054 square feet. The concrete-based structure will not have any accessory parking. Amr Ouda of Jay Architect &amp; Engineering is listed as the architect of record. Demolition permits have not been filed yet for the commercial building on the site. An estimated completion date has not been announced. Subscribe to YIMBY’s daily e-mail Follow YIMBYgram for real-time photo updates Like YIMBY on Facebook Follow YIMBY’s Twitter for the latest in YIMBYnews</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-09-19T15:51:00Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,48 +467,6 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Permits Filed for 149-16 Archer Avenue in Jamaica, Queens</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>https://newyorkyimby.com/2026/09/permits-filed-for-149-16-archer-avenue-in-jamaica-queens.html</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Permits have been filed for a seven-story mixed-use building at 149-16 Archer Avenue in &lt;a href="https://newyorkyimby.com/neighborhoods/jamaica"&gt;Jamaica&lt;/a&gt;, Queens. Located between Sutphin Boulevard and 150th Street, the lot is near the Sutphin Blvd–Archer Avenue–JFK Airport subway station, served by the E, J, and Z trains. Shulem Rabi is listed as the owner behind the applications.</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2026-09-18T10:30:55+00:00</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Fri, 18 Sep 2026 10:30:55 +0000</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>YIMBY</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>YIMBY - Jamaica</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>By: Vanessa Londono 6:30 am on September 18, 2026 Permits have been filed for a seven-story mixed-use building at 149-16 Archer Avenue in Jamaica, Queens. Located between Sutphin Boulevard and 150th Street, the lot is near the Sutphin Blvd–Archer Avenue–JFK Airport subway station, served by the E, J, and Z trains. Shulem Rabi is listed as the owner behind the applications. The proposed 70-foot-tall development will yield 27,127 square feet, with 25,304 square feet designated for residential space and 1,822 square feet for commercial space. The building will have 24 residences, most likely condos based on the average unit scope of 1,054 square feet. The concrete-based structure will not have any accessory parking. Amr Ouda of Jay Architect &amp; Engineering is listed as the architect of record. Demolition permits have not been filed yet for the commercial building on the site. An estimated completion date has not been announced. Subscribe to YIMBY’s daily e-mail Follow YIMBYgram for real-time photo updates Like YIMBY on Facebook Follow YIMBY’s Twitter for the latest in YIMBYnews</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-09-20T16:00:48Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,40 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Joel Steinmetz files plans for 198 units on Jamaica lot, of 297 total</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/joel-steinmetz-files-plans-for-198-units-on-jamaica-block-of-297-total/</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Joel Steinmetz , affiliated with Lead It Builders LLC, filed plans last week for two</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Development 89-52 165th Street, 89-61 164th Street, 89-51 164th Street (Credit - Google Earth) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-09-21T18:12:06Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,34 +473,80 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Joel Steinmetz files plans for 198 units on Jamaica lot, of 297 total</t>
+          <t>56-12 Roosevelt Avenue Nears Topping Out in Woodside, Queens</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/joel-steinmetz-files-plans-for-198-units-on-jamaica-block-of-297-total/</t>
+          <t>https://newyorkyimby.com/2026/09/56-12-roosevelt-avenue-nears-topping-out-in-woodside-queens.html</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Joel Steinmetz , affiliated with Lead It Builders LLC, filed plans last week for two</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
+          <t>Construction is about to top out on 56-12 Roosevelt Avenue, a six-story mixed-use residential building in &lt;a href="https://newyorkyimby.com/neighborhoods/woodside"&gt;Woodside&lt;/a&gt;, Queens. Designed by Xiaohong Zhao of Ameriland Brook LLC for Danny Chang of 5612 Management LLC, the 65-foot-tall structure will span 9,552 square feet and yield nine rental units with an average scope of 764 square feet. The project will also include 2,047 square feet of commercial space, 625 square feet of community facility space, and a 35-foot-long rear yard, according to permits filed last year. The property is located between 56th and 57th Streets.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-09-21T11:30:38+00:00</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Mon, 21 Sep 2026 11:30:38 +0000</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr">
         <is>
+          <t>YIMBY</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>YIMBY - Woodside</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>By: Michael Young and Matt Pruznick 7:30 am on September 21, 2026 Construction is about to top out on 56-12 Roosevelt Avenue, a six-story mixed-use residential building in Woodside, Queens. Designed by Xiaohong Zhao of Ameriland Brook LLC for Danny Chang of 5612 Management LLC, the 65-foot-tall structure will span 9,552 square feet and yield nine rental units with an average scope of 764 square feet. The project will also include 2,047 square feet of commercial space, 625 square feet of community facility space, and a 35-foot-long rear yard, according to permits filed last year. The property is located between 56th and 57th Streets. Crews are tying the rebar for the sixth-story columns and walls and assembling the scaffolding that will support the roof. The bulkhead will extend up the western lot line wall. Façade installation has yet to begin. 56-12 Roosevelt Avenue. Photo by Michael Young. 56-12 Roosevelt Avenue. Photo by Michael Young. 56-12 Roosevelt Avenue. Photo by Michael Young.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>EMP Capital signs $86.5M construction loan with QuadReal for two 99-unit projects in Astoria</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/emp-capital-signs-86-5m-construction-loan-with-quadreal-for-two-99-unit-projects-in-astoria/</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>EMP Capital Group through the entity EMP 37th Street LLC as borrower signed a new</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>NaT</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
           <t>PincusCo</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>PincusCo - Home</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Development 89-52 165th Street, 89-61 164th Street, 89-51 164th Street (Credit - Google Earth) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Chart_Frontpage Transfers 37-09 36th Avenue (l,) at 35-43 37th Street (r.) (Credit - Ralph Kowalczyk architect via DOB) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-09-22T16:53:48Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,86 +467,6 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>56-12 Roosevelt Avenue Nears Topping Out in Woodside, Queens</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>https://newyorkyimby.com/2026/09/56-12-roosevelt-avenue-nears-topping-out-in-woodside-queens.html</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Construction is about to top out on 56-12 Roosevelt Avenue, a six-story mixed-use residential building in &lt;a href="https://newyorkyimby.com/neighborhoods/woodside"&gt;Woodside&lt;/a&gt;, Queens. Designed by Xiaohong Zhao of Ameriland Brook LLC for Danny Chang of 5612 Management LLC, the 65-foot-tall structure will span 9,552 square feet and yield nine rental units with an average scope of 764 square feet. The project will also include 2,047 square feet of commercial space, 625 square feet of community facility space, and a 35-foot-long rear yard, according to permits filed last year. The property is located between 56th and 57th Streets.</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2026-09-21T11:30:38+00:00</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Mon, 21 Sep 2026 11:30:38 +0000</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>YIMBY</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>YIMBY - Woodside</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>By: Michael Young and Matt Pruznick 7:30 am on September 21, 2026 Construction is about to top out on 56-12 Roosevelt Avenue, a six-story mixed-use residential building in Woodside, Queens. Designed by Xiaohong Zhao of Ameriland Brook LLC for Danny Chang of 5612 Management LLC, the 65-foot-tall structure will span 9,552 square feet and yield nine rental units with an average scope of 764 square feet. The project will also include 2,047 square feet of commercial space, 625 square feet of community facility space, and a 35-foot-long rear yard, according to permits filed last year. The property is located between 56th and 57th Streets. Crews are tying the rebar for the sixth-story columns and walls and assembling the scaffolding that will support the roof. The bulkhead will extend up the western lot line wall. Façade installation has yet to begin. 56-12 Roosevelt Avenue. Photo by Michael Young. 56-12 Roosevelt Avenue. Photo by Michael Young. 56-12 Roosevelt Avenue. Photo by Michael Young.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>EMP Capital signs $86.5M construction loan with QuadReal for two 99-unit projects in Astoria</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/emp-capital-signs-86-5m-construction-loan-with-quadreal-for-two-99-unit-projects-in-astoria/</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>EMP Capital Group through the entity EMP 37th Street LLC as borrower signed a new</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>NaT</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Chart_Frontpage Transfers 37-09 36th Avenue (l,) at 35-43 37th Street (r.) (Credit - Ralph Kowalczyk architect via DOB) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here.</t>
         </is>
       </c>
     </row>

</xml_diff>